<commit_message>
Se agregaron más ADR, algunos fueron rechazados o cambiados de una forma en la que se hicieron más fáciles de entender, al final estos pintan un camino claro, y una decisión que me pareció importante es la necesidad de agregar un caché, siguen marcados cómo propuestos, debido a que podría ser útil trabajar información en caché dada la situación
</commit_message>
<xml_diff>
--- a/Documentacion/Drivers-Arquitectonicos/ADR-PoC-Spikes.xlsx
+++ b/Documentacion/Drivers-Arquitectonicos/ADR-PoC-Spikes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juanp\FlorLogic\Documentacion\Drivers-Arquitectonicos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C551A4E8-5CD2-4674-9256-AB0535738F12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9609485A-F13D-4E27-AF9F-1F8D6D02A66D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C1791130-1362-441B-BE9A-13A8318769B9}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="230">
   <si>
     <t>ID</t>
   </si>
@@ -443,6 +443,294 @@
   </si>
   <si>
     <t>No es definitivo, queda abierto para discutir. Mientras tanto, lo que este ADR decidió sigue en pie para el asistente de captura en campo, que es otra cosa. Al escribir el reemplazo hay que decidir tres cosas: qué máquina hace falta, cuánto sube la instalación, y qué tan acotadas quedan las funciones que se le permiten.</t>
+  </si>
+  <si>
+    <t>Separación de deberes entre administrador técnico y administrador de producción</t>
+  </si>
+  <si>
+    <t>Depreciada</t>
+  </si>
+  <si>
+    <t>Había dos respuestas contrarias escritas. Una decía que el administrador de la empresa es el único que puede modificar un registro ya sincronizado. La otra decía que si ese mismo administrador intenta modificar un registro de producción, el sistema debe rechazarlo.</t>
+  </si>
+  <si>
+    <t>Partir el papel de administrador en dos capacidades que nunca coinciden en la misma persona: una técnica, que maneja usuarios, permisos, parámetros y catálogo pero no puede tocar un registro de producción, y otra de producción, que autoriza las correcciones. El intento de la capacidad técnica se rechaza y queda registrado.</t>
+  </si>
+  <si>
+    <t>Resolvía la contradicción del papel, pero no funciona en la finca: la información de producción es cambiante, muy variable y a veces errática, y el administrador de producción necesita poder hacer los cambios necesarios para sacar la producción sin que el sistema se lo impida. Un rechazo de plano por rol convierte una herramienta en un obstáculo.</t>
+  </si>
+  <si>
+    <t>Se deprecia y la sustituye una decisión nueva que controla por la magnitud del cambio y no por el rol: los cambios puntuales se aplican y quedan en la bitácora; los movimientos drásticos piden la confirmación de un segundo administrador, como notificación y no como impedimento. Se conserva esta entrada porque aquí está el razonamiento del problema que había que resolver.</t>
+  </si>
+  <si>
+    <t>El horizonte de las correcciones es el ciclo de producción</t>
+  </si>
+  <si>
+    <t>El catálogo de requisitos y el libro de escenarios se escribieron en momentos distintos y las decisiones posteriores movieron el suelo de los dos. La contradicción más grande era esta: un documento decía que no se conserva el valor anterior a una corrección, y otro decía que nada se sobrescribe nunca. Cada respuesta daba un modelo de datos distinto.</t>
+  </si>
+  <si>
+    <t>Atar la retención de correcciones al ciclo de producción y no al tiempo. Mientras la producción está abierta se guardan todas las modificaciones de sus campos y se puede devolver una corrección al valor anterior. Cuando el administrador declara la actividad terminada, el estado se consolida en el último valor conocido por campo. Al capturador no se le pide nada: ni motivo escrito ni autorización; la autoría viaja sola porque ya está en el registro.</t>
+  </si>
+  <si>
+    <t>Las dos posturas tenían razón sobre horizontes distintos y nadie lo había separado: el cliente rechazaba arrastrar correcciones en la historia larga, que es la que consulta, y la auditoría hace falta mientras el dato todavía se está formando. Y el límite de retención deja de ser una cifra discutible y pasa a ser un hecho del negocio: la producción está cerrada o no lo está.</t>
+  </si>
+  <si>
+    <t>Queda pendiente el trabajo de redacción sobre los requisitos y escenarios que quedaron mal escritos por esta decisión. Eso es una tarea, no una decisión, y no debería seguir viviendo dentro de este ADR.</t>
+  </si>
+  <si>
+    <t>Las decisiones que había que tomar antes de la primera tabla</t>
+  </si>
+  <si>
+    <t>Antes de escribir la primera tabla del dominio había cinco preguntas sin responder, y las cinco eran del equipo y no del cliente.</t>
+  </si>
+  <si>
+    <t>Agruparlas y resolverlas juntas antes de empezar, porque se condicionaban entre ellas: cómo se representa un campo capturado para que sea dato y no columna, cómo se identifica un registro para que sincronizar dos veces no lo duplique, qué es exactamente una sesión de sincronización, si hacían falta tres versionados o uno solo, y dónde corre la inteligencia artificial.</t>
+  </si>
+  <si>
+    <t>Las cinco encarecen enormemente si se toman después de tener instalaciones desplegadas en casa de clientes: cambiarlas más tarde no es reorganizar código, es migrar todas las sedes una por una y sin acceso directo.</t>
+  </si>
+  <si>
+    <t>Se deprecia porque las cinco decisiones ya tienen su propio ADR y esta entrada dejó de decidir nada. Se conserva por el razonamiento de por qué iban juntas. Arrastra un pendiente: los acuerdos que los dos desarrolladores tenían que cerrar antes de escribir código por separado se quedaron sin documento cuando se limpió la carpeta que los contenía, y hay que decidir si vuelven o si ya están cubiertos.</t>
+  </si>
+  <si>
+    <t>Se conserva toda la información de cada producción durante cinco años</t>
+  </si>
+  <si>
+    <t>Se pide poder consultar cinco años en línea, aceptar demora para lo más antiguo, y que el costo no crezca al mismo ritmo que los datos. La respuesta natural sería ir soltando detalle con la edad, pero eso exige saber cuánto hay y qué se consulta de verdad, y hoy no se sabe ninguna de las dos cosas.</t>
+  </si>
+  <si>
+    <t>Conservar absolutamente toda la información de cada producción, sin soltar detalle, durante cinco años: cada modificación de cada campo, con su autor, de las producciones abiertas y de las cerradas por igual. No se construye ninguna política de degradación en la primera entrega. Los cinco años no son un plazo para borrar: son el plazo para decidir con volumen real en la mano.</t>
+  </si>
+  <si>
+    <t>El espacio no es la restricción. Una finca acumula del orden de decenas de gigabytes en cinco años, y como cada empresa tiene su instalación ese volumen no se suma entre clientes: veinte fincas no son un terabyte en un sitio, son veinte servidores modestos. Lo que sí puede apretar es el tiempo de consulta. Y al no degradar, la promesa de que el costo crezca más despacio que los datos pierde su mecanismo principal.</t>
+  </si>
+  <si>
+    <t>Hay que construir desde ya tres cosas aunque hoy no sirvan para nada: el cierre de producción, la política de retención como dato del catálogo y no como código, y la medición de cuánto ocupa y qué se consulta. Sin eso, dentro de cinco años se volvería a decidir a ciegas. Lo único que rompería el cálculo es que algún día entren fotos: una sola imagen pesa más que una producción entera de datos. El tiempo de consulta lo atacan la decisión de totales ya calculados y la separación entre la zona activa y el histórico.</t>
+  </si>
+  <si>
+    <t>El histórico se consulta por totales ya calculados y carga progresiva</t>
+  </si>
+  <si>
+    <t>Al conservarlo todo, el problema deja de ser el espacio y pasa a ser cuánto tarda una consulta que recorre millones de anotaciones.</t>
+  </si>
+  <si>
+    <t>Dos mecanismos, y el orden importa. Primero, la consulta no recorre anotaciones: lee totales ya calculados por los niveles que el negocio usa —finca, bloque, nave, cama, sección, producción, periodo—, y sobre una producción cerrada esos totales no vuelven a cambiar nunca, así que se calculan una vez en el cierre y se leen para siempre. Segundo, la pantalla se sirve en el orden en que la persona navega: primero lo general de la finca y, mientras lee y decide a dónde ir, se traen las categorías que va pidiendo.</t>
+  </si>
+  <si>
+    <t>Lo que la persona nunca abre, no se calcula nunca, y en una consulta exploratoria eso es la mayor parte de la pantalla. Lo que ya se cargó no se va borrando ni descartando: se queda en el caché del navegador mientras dura la consulta, así que volver a la pantalla anterior no vuelve a pedirlo. A cambio, cada pedazo tiene que ser rápido por sí solo: partir una consulta lenta en cinco no la arregla, mueve la espera. Y queda prohibido pedir de a una fila.</t>
+  </si>
+  <si>
+    <t>Esto sirve para explorar, no para extraer: una exportación completa o una auditoría de un lote entero siguen siendo pesadas y van por el camino del trabajo en segundo plano. Y abre la posibilidad de ir más lejos con un caché activo de la producción y la sincronización, que es una decisión aparte y más grande.</t>
+  </si>
+  <si>
+    <t>Cada campo capturado es un hecho; la cama es la unidad de captura</t>
+  </si>
+  <si>
+    <t>Los campos que se capturan tienen que ser datos y no columnas. Si agregar un tipo de labor o de medición exigiera una columna nueva, exigiría cambiar la estructura de la base en todas las instalaciones, dentro de la casa de cada cliente. Y se pide poder ver el último valor conocido de cada campo con la fecha en que se capturó: un campo con fecha propia no puede ser una columna.</t>
+  </si>
+  <si>
+    <t>Cada anotación es una fila, con producción, sección, campo, valor, momento en que entró al sistema, versión del catálogo con la que se validó y, si corrige a otra, a cuál corrige. Agregar una anotación nueva es agregar una fila al catálogo, nunca cambiar la estructura. La estructura geográfica y el catálogo sí son tablas normales; solo el valor va en formato flexible. La persona captura una cama completa de una sentada, aunque el dato aterrice en la sección: nadie captura una sección. Y al cerrar la producción se arma un documento consolidado que ya no cambia.</t>
+  </si>
+  <si>
+    <t>Es la forma más flexible posible y se paga caro: la base de datos deja de validar los tipos —los valida el motor de reglas—, una pantalla de veinte campos es un giro sobre veinte filas, y las filas se multiplican por la cantidad de campos de cada visita. A cambio, dos personas capturando a la vez no chocan, sincronizar sigue siendo insertar sin conflicto, y ninguna pantalla se construye directamente sobre esas filas.</t>
+  </si>
+  <si>
+    <t>Vuelve a propuesta: hay que analizar más a fondo la forma de almacenar la información antes de darla por aceptada. Además la trazabilidad sube al nivel de la captura de la cama, así que cada anotación deja de tener que guardar su propio autor y fecha, y eso cambia la tupla escrita arriba. Cada campo declara en el catálogo a qué niveles se puede anotar y qué pasa al anotarlo por encima de la cama: una fumigación de un lote se hereda a todas sus camas, pero quinientos tallos de un lote no se reparten, porque repartir sería inventar un dato con cara de bueno.</t>
+  </si>
+  <si>
+    <t>Sincronización diaria, y si se pierde un teléfono se recaptura</t>
+  </si>
+  <si>
+    <t>Si el registro vive en el teléfono durante la jornada, quedan dos preguntas: cada cuánto sale la información, y qué se hace cuando un teléfono se pierde o se rompe con capturas dentro.</t>
+  </si>
+  <si>
+    <t>La sincronización apunta a diaria: apenas hay red, y forzable por la persona cuando quiera. El recordatorio se endurece con la antigüedad de lo pendiente: primero avisa, después estorba, después impide seguir trabajando con normalidad. No se construye recuperación de teléfonos, ni reparación ni clonado. En cambio sí se construye la lista exacta de camas que hay que volver a caminar, porque el servidor sabe qué esperaba de ese dispositivo.</t>
+  </si>
+  <si>
+    <t>Convierte una pérdida difusa en una orden de trabajo concreta. Pero la promesa de que recapturar sale más barato solo es cierta si el dato es reciente: a un día se vuelve a caminar la cama y se recuenta; a quince, nadie recuenta unos tallos cortados hace diez días y ya despachados. Si el recordatorio falla o se ignora, el plan de respaldo desaparece con él.</t>
+  </si>
+  <si>
+    <t>El umbral a partir del cual se bloquea es decisión del negocio, no de interfaz, y hay que preguntárselo al cliente. Y no todos los datos se recapturan igual: una siembra o una erradicación se reconstruyen mirando la cama, un corte no, porque se fue con los tallos.</t>
+  </si>
+  <si>
+    <t>Lo asignado es el denominador de lo que falta por capturar</t>
+  </si>
+  <si>
+    <t>Se quiere un tablero que muestre qué está sin capturar y sin sincronizar, pero faltaba decir de dónde sale lo que se espera recibir.</t>
+  </si>
+  <si>
+    <t>Lo esperado viaja en el paquete que baja al teléfono: qué bloques y camas le tocan a ese dispositivo y en qué jornada. Lo esperado menos lo recibido es lo que falta. No hace falta que el teléfono reporte su estado: la ausencia de reporte es la señal.</t>
+  </si>
+  <si>
+    <t>La misma consulta sirve para tres cosas: el avance de la jornada, el aviso de lo que lleva mucho sin sincronizar y la lista de camas a rehacer cuando se pierde un dispositivo. Hay que construir dos tableros distintos y no mezclarlos: el de la empresa ve sus camas con nombre, dispositivo y fechas, porque es su información; el del proveedor ve solo salud y conteos, porque una lista de camas con cifras es información de negocio y no puede salir de la finca.</t>
+  </si>
+  <si>
+    <t>Tiene que poderse cerrar una cama como visitada sin novedad. Si pasar por una cama y no encontrar nada que anotar cuenta como falta, el tablero avisa en falso todos los días y deja de mirarse en dos semanas, y con él se cae el plan de recuperación. Es un toque más en el formulario, así que cambia el tiempo de captura que hay que cronometrar.</t>
+  </si>
+  <si>
+    <t>La identidad del dato y la identidad de la captura son cosas distintas</t>
+  </si>
+  <si>
+    <t>Hacía falta decidir cómo se identifica lo que se anota para que recibirlo dos veces no lo duplique y para poder encadenar las correcciones. Al mirarlo de cerca aparece que los datos puntuales —líneas, tallos, variedad— no necesitan identificar su origen uno por uno: lo que necesita quedar identificado es que ese conjunto de datos de una cama salió de tal captura, y que esa captura está relacionada con tal persona.</t>
+  </si>
+  <si>
+    <t>Separar dos cosas que se le estaban pidiendo al mismo identificador. La identidad técnica de cada anotación es un código único que genera el teléfono al confirmar la captura, sin red; es opaco y solo sirve para que recibir el mismo envío dos veces no lo duplique, así que no se ordena ni se audita por él. Aparte va la clave del hecho —producción, sección, campo y jornada—, que responde si dos anotaciones hablan del mismo dato del mundo. Deliberadamente la clave del hecho no incluye ni el autor ni el dispositivo: si los incluyera, dos personas anotando la misma cama el mismo día serían dos hechos distintos, el choque desaparecería del radar en vez de resolverse, y el error quedaría invisible y con cara de dato bueno.</t>
+  </si>
+  <si>
+    <t>Recibir el mismo envío dos veces no hace nada, que es lo normal porque el teléfono no borra hasta que el servidor confirma. Recibir el mismo identificador con contenido distinto no es un reenvío: es corrupción o un error de programa, así que se rechaza, se registra y se avisa, nunca se sobrescribe. Y dos anotaciones distintas del mismo hecho entran las dos; el sistema decide después cuál es el estado, sin que nadie tenga que mediar.</t>
+  </si>
+  <si>
+    <t>A quién pertenece cada dato no se responde aquí: se responde un nivel más arriba, en la captura de la cama. El prototipo actual contradice esta decisión en cuatro puntos y hay que corregirlo antes de medir sobre él. Falta además definir qué es «la jornada»: el día natural, el turno o la visita son respuestas distintas y las decide el proceso de captura.</t>
+  </si>
+  <si>
+    <t>La captura se identifica cuando llega a la base de datos de la finca</t>
+  </si>
+  <si>
+    <t>Estaba decidido que la trazabilidad no es dato por dato, y sobre esa idea descansa buena parte de la auditoría del sistema. Pero faltaba decir en qué punto y en qué momento queda identificada la información. La captura es el conjunto completo de información que se desea sincronizar, y vive perfectamente dentro del celular durante toda la jornada sin depender de nadie.</t>
+  </si>
+  <si>
+    <t>Esa captura se transporta a la finca, y se identifica y adquiere trazabilidad a partir del momento en que llega a la base de datos principal. El servidor abre el intercambio y deja registrado qué dispositivo lo trajo, qué persona estaba autenticada, la hora de inicio y de fin según su propio reloj, la diferencia entre ese reloj y el del teléfono, con qué versión de configuración venía operando y cuál se le entregó, cuántas anotaciones entraron, cuántas se rechazaron y cómo terminó el intercambio.</t>
+  </si>
+  <si>
+    <t>Es lo que se le enseña a un auditor, y es lo que permite responder con qué reglas estaba operando ese teléfono sin tener que preguntárselo al teléfono. El dato no pierde su origen: se sabe de qué captura salió y con qué persona está relacionada esa captura. Aparece una tabla nueva, pequeña frente al volumen de anotaciones.</t>
+  </si>
+  <si>
+    <t>No confundirla con la sesión de trabajo de la persona dentro de la aplicación, que es otra cosa y sigue abierta; que compartan la palabra es justo por donde se cuela una contradicción nueva. Y ningún intercambio queda abierto para siempre: si se interrumpe, se cierra como parcial con lo que alcanzó a entrar, porque una traza con intercambios abiertos no es una traza.</t>
+  </si>
+  <si>
+    <t>Un solo paquete de configuración por empresa</t>
+  </si>
+  <si>
+    <t>Había tres cosas versionándose por separado —el catálogo, las reglas de validación y los parámetros de cálculo— y cada anotación tenía que guardar con cuál de las tres se validó.</t>
+  </si>
+  <si>
+    <t>Publicarlas juntas como un solo paquete de configuración de la empresa: inmutable, con un único número de versión y distribuido como un solo archivo. La versión de la aplicación queda fuera del paquete: son dos ejes distintos, el del dato y el del código, y se cruzan dentro de cada anotación pero no se fusionan. La asignación diaria de camas tampoco entra, porque cambia todos los días y no puede arrastrar una versión de configuración cada vez.</t>
+  </si>
+  <si>
+    <t>Reproducir una validación pasa de tener que acertar tres versiones —fallando en silencio si se acierta mal— a citar una sola: o es exacto o es imposible, nunca casi. Y demostrar que el teléfono y el servidor entienden lo mismo pasa de ser un problema combinatorio a una lista manejable de casos. El costo honesto es que cambiar un solo parámetro sube toda la versión, así que el paquete lleva un resumen de qué cambió para que la consola no diga «todo cambió» cada vez.</t>
+  </si>
+  <si>
+    <t>Cambiar reglas y normas no es algo que se haga a diario: unas reglas bien definidas para el teléfono probablemente no cambien casi nunca. La flexibilidad no se busca por el uso diario, se busca para poder adaptarse a negocios distintos y para que más adelante sea fácil corregir o agregar una regla que falte o que haya que mejorar. Es una flexibilidad pequeña y deliberada, para que la aplicación pueda crecer y hacerse más a la medida sin tener que republicarla. El número de versión es por empresa: la versión cuarenta y tres de una no tiene ninguna relación con la cuarenta y tres de otra.</t>
+  </si>
+  <si>
+    <t>La inteligencia artificial sugiere en el teléfono y se entrena en el servidor de la finca</t>
+  </si>
+  <si>
+    <t>El asistente de captura se ofreció entrenado con la información del propio cliente, y eso admitía dos lugares: el servidor de la finca, que exigiría hardware especial y encarecería cada instalación, o el propio teléfono, con un modelo pequeño y de alcance limitado.</t>
+  </si>
+  <si>
+    <t>Sugerir corre en el teléfono, sin red, al lado del motor de reglas. Entrenar corre en el servidor de la finca, por lotes y fuera de la jornada. El servidor no lleva hardware de inteligencia artificial, así que el precio de instalación no se mueve.</t>
+  </si>
+  <si>
+    <t>En un caso real de captura la ayuda en el teléfono resulta innecesaria: no es lo que hace falta. Lo que hace falta es ayuda para revisar la información, porque son muchas camas y mucha captura y nadie puede mirarlo todo a mano. La decisión resolvía bien el problema equivocado.</t>
+  </si>
+  <si>
+    <t>Se deprecia y la sustituye una decisión nueva de dos momentos: un modelo local ligero en la finca para reconocer, notificar y ayudar a consultar, y un modelo generativo en línea para lo que el local no puede. Sigue en pie de aquí que no se busca un servidor dedicado a inteligencia artificial profesional.</t>
+  </si>
+  <si>
+    <t>El tiempo del sistema: tres horas distintas y un orden que no cambia</t>
+  </si>
+  <si>
+    <t>Se decidió que cuando dos anotaciones chocan gana la más reciente, de forma automática y sin que nadie medie. Se sabe que el reloj del teléfono puede estar desviado. Y se decidió no bloquear a quien tiene el reloj mal. Cruzadas, esas tres decisiones dan un resultado que nadie había nombrado: el teléfono con el reloj adelantado gana todos los choques, siempre y en silencio, y lo que queda tiene cara de dato bueno.</t>
+  </si>
+  <si>
+    <t>Guardar tres tiempos que no se mezclan nunca. La hora que puso el teléfono, que no se toca jamás y sirve para auditar. Una hora corregida con la desviación conocida de ese teléfono, que es la única que decide quién gana un choque. Y la hora del servidor, que dice cuándo entró al sistema. La desviación se mide en cada sincronización —el servidor ya pone su hora, así que la resta no cuesta nada— y se le devuelve al teléfono para que la lleve en sus capturas siguientes. Si dos anotaciones empatan, se desempata por su identificador.</t>
+  </si>
+  <si>
+    <t>Convierte un sesgo invisible en uno medido y visible, que es todo lo que se puede hacer sin bloquear a la persona en pleno campo. Y garantiza que reconstruir el estado dos veces dé siempre el mismo resultado: sin desempate estable, la misma información podría dar dos estados distintos y nadie lo notaría hasta que un número no cuadre meses después.</t>
+  </si>
+  <si>
+    <t>Esto no convierte la hora en un dato confiable: si el reloj cambió entre la captura y la entrega, la corrección aplicada es una estimación, y por eso la hora original se conserva intacta. Y conviene tener presente la proporción: capturar una cama no es costoso, así que perder la información de una cama —que no se busca y no es lo ideal— no sería un problema mortal ni frenaría la producción. Como la actualización es constante, estos datos no son importantes al nivel de asegurarlos a toda costa: son importantes porque sin ellos no hay nada y porque hay mucho flujo. Lo que de verdad hay que proteger es la capacidad de capturar bien.</t>
+  </si>
+  <si>
+    <t>La corrección se controla por la magnitud del cambio, no por el rol</t>
+  </si>
+  <si>
+    <t>La primera respuesta fue partir el papel de administrador en dos capacidades que nunca coinciden en la misma persona, y rechazar de plano el intento de la capacidad técnica. Eso resuelve la contradicción del papel pero no funciona en la finca: la información de producción es cambiante, muy variable y a veces errática, y el administrador de producción necesita poder hacer los cambios necesarios para sacar la producción sin que el sistema se lo impida. Lo que sí hay que impedir es que una sola persona pueda falsificar información o cambiar algo que no debería.</t>
+  </si>
+  <si>
+    <t>El control no depende de quién es, sino de qué tan drástico es el cambio. Un cambio puntual dentro del desarrollo normal de la producción —corregir un número, un valor definido, el nombre de una variedad— no necesita notificar a nadie: se aplica y queda el registro del cambio en la auditoría, de forma que otro administrador que vaya a trabajar sobre lo mismo pueda entender qué se hizo. Un movimiento drástico —borrar o erradicar una cama completa después de haber sincronizado su captura, eliminar cinco bloques, erradicar zonas enteras— necesita la confirmación de un segundo administrador, sea de producción o técnico. No se bloquea la acción: se pide la confirmación. Son acciones perfectamente válidas dentro del negocio, pero ninguna debería poder hacerla una sola persona.</t>
+  </si>
+  <si>
+    <t>La doble aprobación funciona como notificación, no como impedimento directo, así que la operación nunca se detiene esperando a alguien. A cambio hay que definir qué cuenta como drástico y escribirlo como dato del catálogo y no como código, porque cada empresa puede tener un umbral distinto. Y la bitácora deja de ser solo un registro para el auditor: pasa a ser la forma en que dos administradores se entienden cuando trabajan sobre la misma producción.</t>
+  </si>
+  <si>
+    <t>Sustituye al ADR de separación de deberes, que queda depreciado. Falta escribir la lista de acciones drásticas y decidir qué pasa si el segundo administrador no confirma: si el cambio queda pendiente, si se aplica y se puede revertir, o si caduca. También hay que revisar el requisito que hoy dice que el registro sincronizado solo lo modifica el administrador de la empresa.</t>
+  </si>
+  <si>
+    <t>ADR-033</t>
+  </si>
+  <si>
+    <t>La producción activa vive aparte del histórico por ser un conjunto acotado</t>
+  </si>
+  <si>
+    <t>Rechazada</t>
+  </si>
+  <si>
+    <t>Se propuso separar el almacén en dos zonas por velocidad de acceso, argumentando que lo que está en producción es un conjunto acotado: una finca no podría tener más producciones abiertas que secciones de cama tiene, y por eso ese número no crecería con los años. Lo que sí crecería sin techo sería lo ya cerrado.</t>
+  </si>
+  <si>
+    <t>Separar el almacén en dos zonas. La información activa de producción viviría en una zona de acceso fácil y carga rápida, y lo ya cerrado pasaría a una zona donde puede ser más lento de cargar, siendo el cierre de la producción la frontera entre las dos.</t>
+  </si>
+  <si>
+    <t>Se rechaza porque la premisa no se sostiene. Una finca sí puede tener más producciones que camas ocupadas: se pueden iniciar o planear producciones desde antes, sin estar todavía sobre camas ocupadas, es muy posible que se habiliten más camas para más producciones, y una producción puede crecer porque no tiene un tamaño fijo. La solución no es definir un tamaño de producción, sino poder ofrecer la información activa de forma rápida, y eso se resuelve con el caché delante de la base de datos. Además cae con ella la afirmación de que una finca con ocho años de operación capturaría igual de rápido que el primer día: esa garantía ya no la da la forma del negocio, la tiene que dar el mecanismo.</t>
+  </si>
+  <si>
+    <t>Es una presunción falsa. Se conserva la entrada porque el razonamiento equivocado también es información: el dimensionamiento que se hizo apoyado en el conjunto acotado hay que rehacerlo. Si algo vale la pena conservar de aquí, es una sola línea, y cabe como matiz de la decisión de consulta del histórico: lo cerrado puede permitirse cargar más lento; lo activo no.</t>
+  </si>
+  <si>
+    <t>ADR-034</t>
+  </si>
+  <si>
+    <t>Caché delante de la base de datos con las producciones activas</t>
+  </si>
+  <si>
+    <t>La información activa de producción tiene que poder consultarse rápido, y no se puede apoyar en que el conjunto activo sea pequeño, porque no lo es: se pueden iniciar o planear producciones desde antes, se pueden habilitar más camas, y una producción puede crecer. Además, cuando alguien cambia algo de una producción abierta, ese cambio tendría que viajar y volver por la base de datos para que los demás lo vean.</t>
+  </si>
+  <si>
+    <t>Poner el caché delante de la base de datos, no en el navegador de cada quien, y mantener ahí la información de las producciones activas. La consulta del día a día se sirve desde el caché y toca el almacén lo menos posible. El caché no es una copia ciega: lleva verificaciones y correcciones para que lo que sirve sea lo que hay.</t>
+  </si>
+  <si>
+    <t>Si algo se actualiza en el caché, todos reciben el cambio sin necesidad de una transacción extra que lo envíe desde cada dispositivo, y eso quita de en medio buena parte de los choques posibles. El punto de consulta y el punto de actualización pasan a ser el mismo, así que deja de haber varias versiones de la verdad circulando. A cambio aparece una pieza más que operar en cada instalación, y el problema clásico del caché: hay que decidir cuándo lo guardado deja de ser válido, porque una pantalla que muestra un número viejo con cara de nuevo es peor que una que tarda.</t>
+  </si>
+  <si>
+    <t>Queda como propuesta porque falta afinar el sitio exacto y la forma de invalidar. Lo que ya se cargó en el navegador durante una consulta tampoco se va borrando, pero eso es una comodidad de la pantalla y no el mecanismo: el mecanismo es este caché. Y como el conjunto activo no está acotado, hay que decidir qué entra al caché y qué no cuando una finca tenga muchas producciones abiertas a la vez.</t>
+  </si>
+  <si>
+    <t>ADR-035</t>
+  </si>
+  <si>
+    <t>La sesión de captura es la unidad de trazabilidad</t>
+  </si>
+  <si>
+    <t>Estaba escrito que cada valor anotado lleva su propio autor. Visto de cerca, eso no es lo que hace falta: los datos puntuales —líneas, tallos, variedad— no necesitan identificar su origen uno por uno. Lo que necesita quedar identificado es de qué captura salieron y quién hizo esa captura.</t>
+  </si>
+  <si>
+    <t>La unidad que lleva la trazabilidad es la sesión de captura, y es la que le pone tiempo a los datos: en este momento de captura, esta persona fue la responsable, esta información capturó, y esto es todo lo relacionado con esa sesión. Una sesión de captura no es una sola cama: puede abarcar varias camas, varios bloques, o lo que la persona haya recorrido. Los eventos y datos que se obtuvieron cuelgan de ella en grupos claros, y cada uno sigue diciendo a qué cama, sección o bloque pertenece.</t>
+  </si>
+  <si>
+    <t>Se simplifica mucho lo que hay que guardar en cada valor anotado, y sobre el volumen que se maneja eso no es menor. Y se conserva el camino para llegar al origen, que es lo que importa: cuando una proyección falla, hace falta poder bajar hasta qué cama la desvió y desde ahí subir a qué sesión de captura y qué persona produjo ese dato. Atar la trazabilidad a una sola cama no serviría, sería costoso de consultar; y dejarla suelta en cada dato tampoco. Los grupos claros son lo que hace que ese camino exista.</t>
+  </si>
+  <si>
+    <t>Esto cambia lo que hoy dice la decisión del modelo de datos, que pone autor y fecha de captura en cada anotación por separado. Hay que ajustarla, y es una de las razones por las que esa decisión vuelve a estado de propuesta. Falta decidir cómo se cierra una sesión de captura: si la cierra la persona, si la cierra el envío, o si se corta sola.</t>
+  </si>
+  <si>
+    <t>ADR-036</t>
+  </si>
+  <si>
+    <t>La inteligencia artificial en dos momentos, y es opcional</t>
+  </si>
+  <si>
+    <t>Estaba decidido que la inteligencia artificial sugiriera en el teléfono y se entrenara en el servidor de la finca. En un caso real de captura eso resulta innecesario: el asistente en el teléfono no es lo que hace falta. Lo que sí hace falta es ayuda para revisar la información, porque son muchas camas y mucha captura y nadie puede mirarlo todo a mano.</t>
+  </si>
+  <si>
+    <t>Dos momentos, con dos alcances distintos, y ninguno exige un servidor dedicado a inteligencia artificial profesional. En la finca, un modelo local ligero: un modelo abierto y sencillo, de los que corren en un computador modesto —del orden de 16 GB de memoria—, con una misión muy precisa, que es reconocer, notificar y ayudar a consultar. Sirve para reunir rápido la información rara, contradictoria, desactualizada o que necesita atención, y para trabajar marcando, buscando contradicciones y corrigiendo mientras se rastrea el origen del dato; no se busca generación de documentos grandes, que son muchos más tokens de los que un equipo tan limitado puede manejar. En línea, un modelo generativo de buena calidad para lo que el local no puede: generar documentos, archivos y textos largos. En el teléfono, nada por ahora. Y todo esto es opcional: si el cliente no lo necesita, no lo quiere, o no tiene el equipo para ejecutarlo, no tiene cabida dentro de su finca ni de su sistema.</t>
+  </si>
+  <si>
+    <t>Al ser opcional, el precio base de instalación no se mueve: el computador con memoria suficiente entra solo para quien lo quiera, y se cotiza aparte. El aislamiento entre empresas se cumple por construcción en el momento local, porque el modelo vive dentro de la instalación. El momento en línea es el que hay que revisar con cuidado, porque ahí la información sale de la finca.</t>
+  </si>
+  <si>
+    <t>Sustituye a la decisión de que la IA infiera en el teléfono y se entrene en el nodo, y resuelve el alcance que dejaba abierto el ADR del asistente de captura. Falta decidir qué información puede salir hacia el servicio en línea y con qué autorización, porque el compromiso con el cliente es que su información no sale por ningún canal. Falta también fijar el modelo abierto concreto y medirlo, y acotar por escrito qué se le permite hacer al modelo local.</t>
   </si>
 </sst>
 </file>
@@ -867,7 +1155,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8AD5457-70C5-4508-9A86-7FAFDA9C1359}">
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.44140625" customWidth="1"/>
@@ -985,7 +1273,7 @@
       <c r="E5" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="5" t="s">
         <v>60</v>
       </c>
       <c r="G5" s="4" t="s">
@@ -1258,7 +1546,7 @@
       <c r="D17" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="E17" s="5" t="s">
+      <c r="E17" s="3" t="s">
         <v>120</v>
       </c>
       <c r="F17" s="3" t="s">
@@ -1314,159 +1602,419 @@
         <v>133</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:7" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="4"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B20" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="G20" s="4" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="4"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B21" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="G21" s="4" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="4"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B22" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="144" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="4"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B23" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
-      <c r="G24" s="4"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B24" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="F24" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="G24" s="4" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
-      <c r="E25" s="3"/>
-      <c r="F25" s="3"/>
-      <c r="G25" s="4"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B25" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="72" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="4"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B26" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
-      <c r="G27" s="4"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B27" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="E27" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="F27" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
-      <c r="E28" s="3"/>
-      <c r="F28" s="3"/>
-      <c r="G28" s="4"/>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B28" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
-      <c r="D29" s="3"/>
-      <c r="E29" s="3"/>
-      <c r="F29" s="3"/>
-      <c r="G29" s="4"/>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B29" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B30" s="3"/>
-      <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
-      <c r="E30" s="3"/>
-      <c r="F30" s="3"/>
-      <c r="G30" s="4"/>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B30" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
-      <c r="E31" s="3"/>
-      <c r="F31" s="3"/>
-      <c r="G31" s="4"/>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B31" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="G31" s="4" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="175.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B32" s="3"/>
-      <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
-      <c r="E32" s="3"/>
-      <c r="F32" s="3"/>
-      <c r="G32" s="4"/>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B32" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="G32" s="4" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
-      <c r="D33" s="3"/>
-      <c r="E33" s="3"/>
-      <c r="F33" s="3"/>
-      <c r="G33" s="4"/>
+      <c r="B33" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>201</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="G33" s="4" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="129.6" x14ac:dyDescent="0.3">
+      <c r="A34" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="E34" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="G34" s="4" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A35" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="A36" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="G36" s="4" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="144" x14ac:dyDescent="0.3">
+      <c r="A37" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="G37" s="4" t="s">
+        <v>229</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
A partir de ahora se va a trabajar el diagrama en archivos tipo drawio desde las carpetas del repositorio, los diagramas que no cuentan con color fueron una especulación previa a lo que se iba a desarrollar sin embargo no tiene el formato C4 necesario, pero es una buena base, sin embargo estos modelos no tienen los últimos ADR
</commit_message>
<xml_diff>
--- a/Documentacion/Drivers-Arquitectonicos/ADR-PoC-Spikes.xlsx
+++ b/Documentacion/Drivers-Arquitectonicos/ADR-PoC-Spikes.xlsx
@@ -322,7 +322,7 @@
     <t>Almacenar la información de forma distinta según su antigüedad</t>
   </si>
   <si>
-    <t>Deprecada</t>
+    <t>Depreciada</t>
   </si>
   <si>
     <t>Se había decidido que la información de una producción se guardara de forma distinta según su antigüedad: completa mientras la producción está abierta, resumida cuando ya es reciente, y solo con su resultado cuando es antigua, sin borrar nunca el hecho de producción.</t>
@@ -430,7 +430,7 @@
     <t>El asistente de captura no se compromete hasta medirlo</t>
   </si>
   <si>
-    <t>En revisión — probablemente depreciada</t>
+    <t>Depreciada</t>
   </si>
   <si>
     <t>Este ADR se escribió para no comprometer un asistente que ayudara a llenar el formulario en campo, que el cliente nunca pidió y que era idea de los desarrolladores. Para ese alcance concreto sigue siendo válido. Pero la idea de inteligencia artificial dentro del producto cambió de forma: ya no se piensa como un ayudante para teclear menos, sino como apoyo constante para revisar la información y como recopilador de información más detallada.</t>

</xml_diff>

<commit_message>
AJSDKLAJSD Se me olvidó guardar el nuevo ADR entonces todavía no figuraba en la versión anterior y tampoco cuando se mencionó,
</commit_message>
<xml_diff>
--- a/Documentacion/Drivers-Arquitectonicos/ADR-PoC-Spikes.xlsx
+++ b/Documentacion/Drivers-Arquitectonicos/ADR-PoC-Spikes.xlsx
@@ -1,20 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juanp\FlorLogic\Documentacion\Drivers-Arquitectonicos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9609485A-F13D-4E27-AF9F-1F8D6D02A66D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1747D32-8878-41F2-AD3E-F0654FC6E62F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C1791130-1362-441B-BE9A-13A8318769B9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C1791130-1362-441B-BE9A-13A8318769B9}"/>
   </bookViews>
   <sheets>
     <sheet name="ADR" sheetId="1" r:id="rId1"/>
-    <sheet name="PoC's" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="234">
   <si>
     <t>ID</t>
   </si>
@@ -172,12 +171,6 @@
   </si>
   <si>
     <t>Un único artefacto y lugar dónde trabajar y respaldar, con prioridad Offline-First que es totalmente imoprtate en el negocio, sin embargo, es necesario escalar las capacidades de la solución a las capacidad técnologicas que haya en el dispositivo del cliente.</t>
-  </si>
-  <si>
-    <t>Titulo</t>
-  </si>
-  <si>
-    <t>Problem</t>
   </si>
   <si>
     <t>Se añadió la desisción de evitar SaaS a esta desición de entrega debido a que hubo problemas con el concepto SaaS precisamente por una petición con el cliente reflejada en el ESC-059, escenario que no podría ser cumplido con un modelo de entrega SaaS</t>
@@ -731,6 +724,24 @@
   </si>
   <si>
     <t>Sustituye a la decisión de que la IA infiera en el teléfono y se entrene en el nodo, y resuelve el alcance que dejaba abierto el ADR del asistente de captura. Falta decidir qué información puede salir hacia el servicio en línea y con qué autorización, porque el compromiso con el cliente es que su información no sale por ningún canal. Falta también fijar el modelo abierto concreto y medirlo, y acotar por escrito qué se le permite hacer al modelo local.</t>
+  </si>
+  <si>
+    <t>ADR-037</t>
+  </si>
+  <si>
+    <t>El backend de la finca no tiene lenguaje elegido, y es la pieza de la que cuelga todo lo demás: recibe lo capturado, aplica las reglas, calcula la proyección, responde las consultas y produce los documentos.</t>
+  </si>
+  <si>
+    <t>Java como lenguaje del backend de la finca</t>
+  </si>
+  <si>
+    <t>El backend se construye en Java optando por esta opción debido a los resultados del Spike SPK-017 dónde se muestra la nula divergencia de información importante para el sistema con ejemplos, además el entorno es el más completo para los componentes necesarios para el desarrollo del sistema.</t>
+  </si>
+  <si>
+    <t>Se fácilita la desición de herramientas para demás componentes del sistema, se obtiene una gran disponibilidad del servicio y una estructura basada en objetos que ya había sido definida, no compromete que la lectura de información sea directamente a través de windows por estar en Access, El sistema vuelve su arranque más lento, y aumenta el espacio del aplicativo. ofrece mejor trazabilidad de errores para soporte es conocido por las personas que lo van a desarrollar. fácilita las desiciones.</t>
+  </si>
+  <si>
+    <t>Esta decisión no elige el armazón sobre el que se construye el servicio. Esa elección cambia la memoria que consume el nodo casi a la mitad, y no está medida. Se decide aparte. Junto con cómo se empaqueta ni tampoco cambia las desiciones del disitivo de campo</t>
   </si>
 </sst>
 </file>
@@ -1155,7 +1166,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8AD5457-70C5-4508-9A86-7FAFDA9C1359}">
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.44140625" customWidth="1"/>
@@ -1210,7 +1221,7 @@
         <v>43</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -1218,22 +1229,22 @@
         <v>7</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="G3" s="4" t="s">
         <v>49</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -1241,19 +1252,19 @@
         <v>8</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>53</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>55</v>
       </c>
       <c r="G4" s="4"/>
     </row>
@@ -1262,22 +1273,22 @@
         <v>9</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="F5" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="G5" s="4" t="s">
         <v>59</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
@@ -1285,22 +1296,22 @@
         <v>10</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>40</v>
       </c>
       <c r="D6" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="G6" s="4" t="s">
         <v>74</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -1308,22 +1319,22 @@
         <v>11</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="F7" s="3" t="s">
+      <c r="G7" s="4" t="s">
         <v>65</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
@@ -1331,22 +1342,22 @@
         <v>12</v>
       </c>
       <c r="B8" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D8" s="3" t="s">
+      <c r="F8" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="G8" s="4" t="s">
         <v>70</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
@@ -1354,22 +1365,22 @@
         <v>13</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="D9" s="3" t="s">
+      <c r="F9" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="G9" s="4" t="s">
         <v>79</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -1377,22 +1388,22 @@
         <v>14</v>
       </c>
       <c r="B10" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="E10" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="D10" s="3" t="s">
+      <c r="F10" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="G10" s="4" t="s">
         <v>84</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="115.2" x14ac:dyDescent="0.3">
@@ -1400,22 +1411,22 @@
         <v>15</v>
       </c>
       <c r="B11" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="E11" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="D11" s="3" t="s">
+      <c r="F11" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="G11" s="4" t="s">
         <v>89</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -1423,22 +1434,22 @@
         <v>16</v>
       </c>
       <c r="B12" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="E12" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="F12" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="G12" s="4" t="s">
         <v>95</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
@@ -1446,22 +1457,22 @@
         <v>17</v>
       </c>
       <c r="B13" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="E13" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="C13" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D13" s="3" t="s">
+      <c r="F13" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="G13" s="4" t="s">
         <v>100</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -1469,22 +1480,22 @@
         <v>18</v>
       </c>
       <c r="B14" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="E14" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="C14" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D14" s="3" t="s">
+      <c r="F14" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="G14" s="4" t="s">
         <v>105</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="115.2" x14ac:dyDescent="0.3">
@@ -1492,22 +1503,22 @@
         <v>19</v>
       </c>
       <c r="B15" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E15" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C15" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D15" s="3" t="s">
+      <c r="F15" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="G15" s="4" t="s">
         <v>110</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -1515,22 +1526,22 @@
         <v>20</v>
       </c>
       <c r="B16" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="E16" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="C16" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D16" s="3" t="s">
+      <c r="F16" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="G16" s="4" t="s">
         <v>115</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
@@ -1538,22 +1549,22 @@
         <v>21</v>
       </c>
       <c r="B17" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="E17" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="C17" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D17" s="3" t="s">
+      <c r="F17" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="G17" s="4" t="s">
         <v>120</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="G17" s="4" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -1561,22 +1572,22 @@
         <v>22</v>
       </c>
       <c r="B18" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="E18" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="C18" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D18" s="3" t="s">
+      <c r="F18" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="G18" s="4" t="s">
         <v>125</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="G18" s="4" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
@@ -1584,22 +1595,22 @@
         <v>23</v>
       </c>
       <c r="B19" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="D19" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="E19" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="F19" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="G19" s="4" t="s">
         <v>131</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="G19" s="4" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="115.2" x14ac:dyDescent="0.3">
@@ -1607,22 +1618,22 @@
         <v>24</v>
       </c>
       <c r="B20" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="D20" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="E20" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="F20" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="G20" s="4" t="s">
         <v>137</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="G20" s="4" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
@@ -1630,22 +1641,22 @@
         <v>25</v>
       </c>
       <c r="B21" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E21" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="C21" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D21" s="3" t="s">
+      <c r="F21" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="G21" s="4" t="s">
         <v>142</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="G21" s="4" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="115.2" x14ac:dyDescent="0.3">
@@ -1653,22 +1664,22 @@
         <v>26</v>
       </c>
       <c r="B22" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="E22" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="C22" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="D22" s="3" t="s">
+      <c r="F22" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="G22" s="4" t="s">
         <v>147</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="G22" s="4" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="144" x14ac:dyDescent="0.3">
@@ -1676,22 +1687,22 @@
         <v>27</v>
       </c>
       <c r="B23" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="E23" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="C23" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D23" s="3" t="s">
+      <c r="F23" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="G23" s="4" t="s">
         <v>152</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="G23" s="4" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
@@ -1699,22 +1710,22 @@
         <v>28</v>
       </c>
       <c r="B24" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E24" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="C24" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D24" s="3" t="s">
+      <c r="F24" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="G24" s="4" t="s">
         <v>157</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="G24" s="4" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="158.4" x14ac:dyDescent="0.3">
@@ -1722,22 +1733,22 @@
         <v>29</v>
       </c>
       <c r="B25" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="E25" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="C25" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="D25" s="3" t="s">
+      <c r="F25" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="E25" s="3" t="s">
+      <c r="G25" s="4" t="s">
         <v>162</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="G25" s="4" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="72" x14ac:dyDescent="0.3">
@@ -1745,22 +1756,22 @@
         <v>30</v>
       </c>
       <c r="B26" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="E26" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="C26" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D26" s="3" t="s">
+      <c r="F26" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="E26" s="3" t="s">
+      <c r="G26" s="4" t="s">
         <v>167</v>
-      </c>
-      <c r="F26" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="G26" s="4" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
@@ -1768,22 +1779,22 @@
         <v>31</v>
       </c>
       <c r="B27" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="E27" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="C27" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D27" s="3" t="s">
+      <c r="F27" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="E27" s="3" t="s">
+      <c r="G27" s="4" t="s">
         <v>172</v>
-      </c>
-      <c r="F27" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="G27" s="4" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
@@ -1791,22 +1802,22 @@
         <v>32</v>
       </c>
       <c r="B28" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E28" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="C28" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D28" s="3" t="s">
+      <c r="F28" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="E28" s="3" t="s">
+      <c r="G28" s="4" t="s">
         <v>177</v>
-      </c>
-      <c r="F28" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="G28" s="4" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="115.2" x14ac:dyDescent="0.3">
@@ -1814,22 +1825,22 @@
         <v>33</v>
       </c>
       <c r="B29" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="E29" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="C29" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D29" s="3" t="s">
+      <c r="F29" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="E29" s="3" t="s">
+      <c r="G29" s="4" t="s">
         <v>182</v>
-      </c>
-      <c r="F29" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="G29" s="4" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="172.8" x14ac:dyDescent="0.3">
@@ -1837,22 +1848,22 @@
         <v>34</v>
       </c>
       <c r="B30" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="E30" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="C30" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D30" s="3" t="s">
+      <c r="F30" s="3" t="s">
         <v>186</v>
       </c>
-      <c r="E30" s="3" t="s">
+      <c r="G30" s="4" t="s">
         <v>187</v>
-      </c>
-      <c r="F30" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="G30" s="4" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="86.4" x14ac:dyDescent="0.3">
@@ -1860,22 +1871,22 @@
         <v>35</v>
       </c>
       <c r="B31" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="E31" s="3" t="s">
         <v>190</v>
       </c>
-      <c r="C31" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="D31" s="3" t="s">
+      <c r="F31" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="E31" s="3" t="s">
+      <c r="G31" s="4" t="s">
         <v>192</v>
-      </c>
-      <c r="F31" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="G31" s="4" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="175.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -1883,22 +1894,22 @@
         <v>36</v>
       </c>
       <c r="B32" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="E32" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="C32" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D32" s="3" t="s">
+      <c r="F32" s="3" t="s">
         <v>196</v>
       </c>
-      <c r="E32" s="3" t="s">
+      <c r="G32" s="4" t="s">
         <v>197</v>
-      </c>
-      <c r="F32" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="G32" s="4" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="129.6" x14ac:dyDescent="0.3">
@@ -1906,139 +1917,141 @@
         <v>37</v>
       </c>
       <c r="B33" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="E33" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="C33" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D33" s="3" t="s">
+      <c r="F33" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="E33" s="3" t="s">
+      <c r="G33" s="4" t="s">
         <v>202</v>
-      </c>
-      <c r="F33" s="3" t="s">
-        <v>203</v>
-      </c>
-      <c r="G33" s="4" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A34" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="C34" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="B34" s="3" t="s">
+      <c r="D34" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="C34" s="3" t="s">
+      <c r="E34" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="D34" s="3" t="s">
+      <c r="F34" s="3" t="s">
         <v>208</v>
       </c>
-      <c r="E34" s="3" t="s">
+      <c r="G34" s="4" t="s">
         <v>209</v>
-      </c>
-      <c r="F34" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="G34" s="4" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="B35" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D35" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="E35" s="3" t="s">
         <v>213</v>
       </c>
-      <c r="C35" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="D35" s="3" t="s">
+      <c r="F35" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="E35" s="3" t="s">
+      <c r="G35" s="4" t="s">
         <v>215</v>
-      </c>
-      <c r="F35" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="G35" s="4" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D36" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="B36" s="3" t="s">
+      <c r="E36" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="C36" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D36" s="3" t="s">
+      <c r="F36" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="E36" s="3" t="s">
+      <c r="G36" s="4" t="s">
         <v>221</v>
-      </c>
-      <c r="F36" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="G36" s="4" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="37" spans="1:7" ht="144" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D37" s="3" t="s">
         <v>224</v>
       </c>
-      <c r="B37" s="3" t="s">
+      <c r="E37" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="C37" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="D37" s="3" t="s">
+      <c r="F37" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="E37" s="3" t="s">
+      <c r="G37" s="4" t="s">
         <v>227</v>
       </c>
-      <c r="F37" s="3" t="s">
+    </row>
+    <row r="38" spans="1:7" ht="99.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="G37" s="4" t="s">
+      <c r="B38" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D38" s="3" t="s">
         <v>229</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="G38" s="4" t="s">
+        <v>233</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{087DBBD2-C328-44AF-AE35-22DB9F92DD22}">
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>44</v>
-      </c>
-      <c r="C1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>